<commit_message>
05 06 oofice last
</commit_message>
<xml_diff>
--- a/test_file2.xlsx
+++ b/test_file2.xlsx
@@ -484,15 +484,11 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>$1,200.00</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>$0.00</t>
-        </is>
+      <c r="A2" t="n">
+        <v>1200</v>
+      </c>
+      <c r="B2" t="n">
+        <v>0</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -504,10 +500,8 @@
           <t>no intraest</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
+      <c r="E2" t="n">
+        <v>9</v>
       </c>
       <c r="F2" t="n">
         <v>1248</v>
@@ -515,30 +509,20 @@
       <c r="G2" t="n">
         <v>1194</v>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>$132.66</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>$1,247.97</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>$0.00</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>0.00</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>$133.33</t>
-        </is>
+      <c r="H2" t="n">
+        <v>133</v>
+      </c>
+      <c r="I2" t="n">
+        <v>1248</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="n">
+        <v>133</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>

</xml_diff>